<commit_message>
Rename to Lumi Trade; clients complete company details on first sign-in
</commit_message>
<xml_diff>
--- a/test/files/filled-template.xlsx
+++ b/test/files/filled-template.xlsx
@@ -300,7 +300,7 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>Highs Business</author>
+    <author>Lumi Trade</author>
   </authors>
   <commentList>
     <comment ref="B4" authorId="0" shapeId="0">
@@ -330,7 +330,7 @@
 <file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>Highs Business</author>
+    <author>Lumi Trade</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
@@ -706,7 +706,7 @@
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Highs Business — Supplier product form  /  供应商产品信息表</t>
+          <t>Lumi Trade — Supplier product form  /  供应商产品信息表</t>
         </is>
       </c>
     </row>

</xml_diff>